<commit_message>
fix(dengue): codigo 4112801 e Joaquim Tavora, nao Jacarezinho
O municipio de codigo IBGE 4112801 estava rotulado como Jacarezinho (que e 4111803).
Casos e populacao sempre foram de Joaquim Tavora; so o nome muda, nas tres
planilhas, no gerar.py, no README dos dados, nos slides da A56 e da A58, na
rubrica da Av01-T3 e na semana16. Nenhum numero mudou. dist/ e o site publicado
so mudam com novo build e deploy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aulas/09set/A55_UC01_11set/public/dados/dengue_pr_bruto.xlsx
+++ b/aulas/09set/A55_UC01_11set/public/dados/dengue_pr_bruto.xlsx
@@ -6047,7 +6047,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -6079,7 +6079,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -6109,7 +6109,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -6139,7 +6139,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -6171,7 +6171,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -6201,7 +6201,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -6233,7 +6233,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -6263,7 +6263,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -6293,7 +6293,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -6327,7 +6327,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -6359,7 +6359,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -6389,7 +6389,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -6419,7 +6419,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -6449,7 +6449,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -6481,7 +6481,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -6513,7 +6513,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -6545,7 +6545,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -6577,7 +6577,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -6607,7 +6607,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -6637,7 +6637,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -6669,7 +6669,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -6701,7 +6701,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -6735,7 +6735,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -6765,7 +6765,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Jacarezinho</t>
+          <t>Joaquim Távora</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -6795,7 +6795,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>TOTAL Jacarezinho</t>
+          <t>TOTAL Joaquim Távora</t>
         </is>
       </c>
       <c r="B210" t="inlineStr"/>

</xml_diff>